<commit_message>
Daily EOD data and reports for 2026-10-29
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261029.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261029.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.637</v>
+        <v>1.64</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.008</v>
+        <v>-0.005</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>250757.3</v>
+        <v>251216.84</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-1225.45</v>
+        <v>-765.91</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.48</v>
+        <v>2.51</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>173600</v>
+        <v>175700</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1400</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>57.56</v>
+        <v>57.52</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.48</v>
+        <v>-0.52</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.90%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>460480</v>
+        <v>460160</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-3840</v>
+        <v>-4160</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>165.52</v>
+        <v>166.39</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2.51</v>
+        <v>3.38</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>1.23%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8150</v>
+        <v>8200</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>197.33</v>
+        <v>197.5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.23</v>
+        <v>0.4</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>789320</v>
+        <v>790000</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>920</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0</v>
+        <v>0.215</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.21</v>
+        <v>0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>2.38%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>4300</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.82</v>
+        <v>11.77</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>35991.9</v>
+        <v>35839.65</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>456.75</v>
+        <v>304.5</v>
       </c>
     </row>
     <row r="13">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.079</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.079</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>474</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-474</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.2</v>
+        <v>37.21</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.83%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.73</v>
+        <v>32.74</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42156.24</v>
+        <v>42169.12</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>772.8</v>
+        <v>785.6799999999999</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1761457.08</v>
+        <v>1769061.26</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-7486.4</v>
+        <v>117.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>